<commit_message>
Reorganização do código em POO (Programa Orientada a Objetos) - Parte 2
</commit_message>
<xml_diff>
--- a/Dados de Entrada/database_yield_curves.xlsx
+++ b/Dados de Entrada/database_yield_curves.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a69383772dadf60a/Documentos/Vitor/Projetos/PycharmProjects/Projeto_TotalEnergies/Dados de Entrada/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="277" documentId="8_{16656DA0-1CDE-44F6-84C5-B306D7FC66E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2CAB174-DE66-487B-8C87-F183A3CA37C6}"/>
+  <xr:revisionPtr revIDLastSave="286" documentId="8_{16656DA0-1CDE-44F6-84C5-B306D7FC66E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA8ED16E-1FDB-49B3-9BC2-FEDC774803B5}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="785" activeTab="8" xr2:uid="{0506B892-8FEF-410F-A807-A4815D37E0A7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="785" firstSheet="15" activeTab="20" xr2:uid="{0506B892-8FEF-410F-A807-A4815D37E0A7}"/>
   </bookViews>
   <sheets>
     <sheet name="MODELO" sheetId="18" r:id="rId1"/>
@@ -1115,12 +1115,6 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1129,6 +1123,12 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1604,36 +1604,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1821,24 +1821,24 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
     </row>
@@ -1847,24 +1847,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>
@@ -1964,7 +1964,7 @@
       <c r="E4" s="10">
         <v>0</v>
       </c>
-      <c r="K4" s="40">
+      <c r="K4" s="38">
         <v>5.4135353387706701E-3</v>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       <c r="E5" s="10">
         <v>0</v>
       </c>
-      <c r="K5" s="41">
+      <c r="K5" s="39">
         <v>4.3984938326937202E-3</v>
       </c>
     </row>
@@ -1998,7 +1998,7 @@
       <c r="E6" s="10">
         <v>0</v>
       </c>
-      <c r="K6" s="41">
+      <c r="K6" s="39">
         <v>4.7368280945150696E-3</v>
       </c>
     </row>
@@ -2015,7 +2015,7 @@
       <c r="E7" s="10">
         <v>0</v>
       </c>
-      <c r="K7" s="41">
+      <c r="K7" s="39">
         <v>1.8608997476545399E-3</v>
       </c>
     </row>
@@ -2032,7 +2032,7 @@
       <c r="E8" s="10">
         <v>1.1841989568344099E-3</v>
       </c>
-      <c r="K8" s="41">
+      <c r="K8" s="39">
         <v>3.0450987044889498E-3</v>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
       <c r="E9" s="10">
         <v>7.9511165169389008E-3</v>
       </c>
-      <c r="K9" s="41">
+      <c r="K9" s="39">
         <v>9.8120162645934407E-3</v>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       <c r="E10" s="10">
         <v>2.1992482070339457E-2</v>
       </c>
-      <c r="K10" s="42">
+      <c r="K10" s="40">
         <v>2.3853381817993999E-2</v>
       </c>
     </row>
@@ -2077,50 +2077,50 @@
       <c r="E11" s="10">
         <v>3.2142858410496258E-2</v>
       </c>
-      <c r="K11" s="42">
+      <c r="K11" s="40">
         <v>3.40037581581508E-2</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.80042009748954401</v>
       </c>
       <c r="E12" s="10">
         <v>4.3308276256729859E-2</v>
       </c>
-      <c r="K12" s="42">
+      <c r="K12" s="40">
         <v>4.5169176004384401E-2</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.85084025909163996</v>
       </c>
       <c r="E13" s="10">
         <v>4.3308276256729859E-2</v>
       </c>
-      <c r="K13" s="42">
+      <c r="K13" s="40">
         <v>4.5169176004384401E-2</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.90042009748954399</v>
       </c>
       <c r="E14" s="10">
         <v>5.3966170123207362E-2</v>
       </c>
-      <c r="K14" s="42">
+      <c r="K14" s="40">
         <v>5.5827069870861903E-2</v>
       </c>
     </row>
@@ -2129,24 +2129,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>
@@ -2332,24 +2332,24 @@
       <c r="E11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
     </row>
@@ -2358,24 +2358,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>
@@ -2561,24 +2561,24 @@
       <c r="E11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
     </row>
@@ -2587,24 +2587,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>
@@ -2790,24 +2790,24 @@
       <c r="E11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
     </row>
@@ -2816,24 +2816,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>
@@ -3080,10 +3080,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.8</v>
       </c>
@@ -3098,10 +3098,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.85</v>
       </c>
@@ -3116,8 +3116,8 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.9</v>
       </c>
@@ -3136,24 +3136,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>207</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>
@@ -3376,10 +3376,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.8</v>
       </c>
@@ -3391,10 +3391,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.85</v>
       </c>
@@ -3406,8 +3406,8 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.9</v>
       </c>
@@ -3423,24 +3423,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>207</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>
@@ -3643,10 +3643,10 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.93203539120356504</v>
       </c>
@@ -3656,10 +3656,10 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.95433625694392898</v>
       </c>
@@ -3669,8 +3669,8 @@
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
@@ -3680,24 +3680,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>
@@ -3900,10 +3900,10 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.61769908564757103</v>
       </c>
@@ -3913,10 +3913,10 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.62725662268490101</v>
       </c>
@@ -3926,8 +3926,8 @@
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.641061962963278</v>
       </c>
@@ -3945,10 +3945,10 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8">
         <v>0.66442475925887601</v>
       </c>
@@ -3957,10 +3957,10 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8">
         <v>0.67292036574097103</v>
       </c>
@@ -3969,8 +3969,8 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8">
         <v>0.68566369444400499</v>
       </c>
@@ -4317,10 +4317,10 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.86088490972131904</v>
       </c>
@@ -4330,10 +4330,10 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.92460171527670498</v>
       </c>
@@ -4343,8 +4343,8 @@
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.94796459259241195</v>
       </c>
@@ -4358,24 +4358,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>
@@ -6517,10 +6517,10 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.92509363295880098</v>
       </c>
@@ -6530,30 +6530,30 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>114</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>115</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -6742,10 +6742,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.95454545454545403</v>
       </c>
@@ -6754,30 +6754,30 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -6958,36 +6958,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>65</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -7176,10 +7176,10 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.84566209727512098</v>
       </c>
@@ -7188,10 +7188,10 @@
       </c>
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.89223742256077898</v>
       </c>
@@ -7200,8 +7200,8 @@
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.93333331010838905</v>
       </c>
@@ -7218,20 +7218,20 @@
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -7412,36 +7412,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -7630,10 +7630,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.93205568021623897</v>
       </c>
@@ -7642,10 +7642,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.95505216032784601</v>
       </c>
@@ -7654,24 +7654,24 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -7862,10 +7862,10 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.86202088008108901</v>
       </c>
@@ -7874,10 +7874,10 @@
       </c>
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.925783920163051</v>
       </c>
@@ -7886,8 +7886,8 @@
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.94878040027465804</v>
       </c>
@@ -7897,20 +7897,20 @@
       <c r="F14" s="8"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -8099,10 +8099,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.774457399130554</v>
       </c>
@@ -8111,10 +8111,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.87262102047161305</v>
       </c>
@@ -8123,8 +8123,8 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.87262102047161305</v>
       </c>
@@ -8133,20 +8133,20 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -8327,36 +8327,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -8545,36 +8545,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -8749,36 +8749,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -8959,36 +8959,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -9185,10 +9185,10 @@
       <c r="K11" s="8"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.87306019120053269</v>
       </c>
@@ -9198,10 +9198,10 @@
       <c r="K12" s="8"/>
     </row>
     <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.93164778021895833</v>
       </c>
@@ -9211,8 +9211,8 @@
       <c r="K13" s="8"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.93164778021895833</v>
       </c>
@@ -9222,20 +9222,20 @@
       <c r="K14" s="8"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -9423,36 +9423,36 @@
       <c r="K10" s="8"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -9627,36 +9627,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -9825,36 +9825,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -10043,38 +10043,38 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -10263,10 +10263,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.87725631768953005</v>
       </c>
@@ -10275,10 +10275,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.87725631768953005</v>
       </c>
@@ -10287,26 +10287,26 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -10475,36 +10475,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -10693,10 +10693,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.87522603978300095</v>
       </c>
@@ -10705,32 +10705,32 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -10906,36 +10906,36 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>98</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -11123,36 +11123,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -11327,36 +11327,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -11541,36 +11541,36 @@
       <c r="E11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -11739,36 +11739,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -11949,36 +11949,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -12167,10 +12167,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.64521739130434697</v>
       </c>
@@ -12179,10 +12179,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.64521739130434697</v>
       </c>
@@ -12191,8 +12191,8 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.75652173913043397</v>
       </c>
@@ -12209,10 +12209,10 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8">
         <v>0.87478260869565205</v>
       </c>
@@ -12221,10 +12221,10 @@
       </c>
     </row>
     <row r="17" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="K17" s="37">
         <v>0.99826086956521698</v>
       </c>
@@ -12233,8 +12233,8 @@
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -12431,10 +12431,10 @@
       <c r="K11" s="8"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.76</v>
       </c>
@@ -12444,10 +12444,10 @@
       <c r="K12" s="8"/>
     </row>
     <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>98</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.75826086956521699</v>
       </c>
@@ -12457,8 +12457,8 @@
       <c r="K13" s="8"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.87652173913043396</v>
       </c>
@@ -12477,23 +12477,23 @@
       <c r="K15" s="8"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="K16" s="8"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>111</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -12682,10 +12682,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.80585009140767805</v>
       </c>
@@ -12694,10 +12694,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.85521023765996296</v>
       </c>
@@ -12706,8 +12706,8 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.9</v>
       </c>
@@ -12716,20 +12716,20 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>120</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -12918,10 +12918,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.80630630630630595</v>
       </c>
@@ -12930,10 +12930,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.85495495495495499</v>
       </c>
@@ -12942,8 +12942,8 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.89909909909909902</v>
       </c>
@@ -12952,20 +12952,20 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>120</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -13157,10 +13157,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.84972577696526497</v>
       </c>
@@ -13169,30 +13169,30 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>123</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -13364,36 +13364,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>123</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -13581,10 +13581,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.59926200863547896</v>
       </c>
@@ -13593,10 +13593,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.65153752697560796</v>
       </c>
@@ -13605,8 +13605,8 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.69950797447615798</v>
       </c>
@@ -13623,10 +13623,10 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8">
         <v>0.74993850267467499</v>
       </c>
@@ -13635,10 +13635,10 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8">
         <v>0.799138990524208</v>
       </c>
@@ -13647,8 +13647,8 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8">
         <v>0.85018446851535401</v>
       </c>
@@ -13854,10 +13854,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.79853747714807999</v>
       </c>
@@ -13866,30 +13866,30 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>123</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -14049,36 +14049,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -14244,36 +14244,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>129</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -14473,10 +14473,10 @@
       <c r="K11" s="8"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>3.1210191082802499E-2</v>
       </c>
@@ -14486,10 +14486,10 @@
       <c r="K12" s="8"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>6.2258064516129002E-2</v>
       </c>
@@ -14499,8 +14499,8 @@
       <c r="K13" s="8"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.124838709677419</v>
       </c>
@@ -14519,20 +14519,20 @@
       <c r="K15" s="8"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -14724,36 +14724,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -14945,10 +14945,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.13677419354838699</v>
       </c>
@@ -14957,10 +14957,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.203870967741935</v>
       </c>
@@ -14969,24 +14969,24 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -15178,10 +15178,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.21</v>
       </c>
@@ -15190,30 +15190,30 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -15391,36 +15391,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -15598,36 +15598,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -15819,10 +15819,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.20499999999999999</v>
       </c>
@@ -15831,30 +15831,30 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -16042,24 +16042,24 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
     </row>
@@ -16068,24 +16068,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>
@@ -16239,36 +16239,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -16460,10 +16460,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.13107752956636001</v>
       </c>
@@ -16472,10 +16472,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.196452036793692</v>
       </c>
@@ -16484,24 +16484,24 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -16693,10 +16693,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.136005256241787</v>
       </c>
@@ -16705,30 +16705,30 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -16906,36 +16906,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -17127,10 +17127,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.75</v>
       </c>
@@ -17139,10 +17139,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.8</v>
       </c>
@@ -17151,8 +17151,8 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.89999999999999902</v>
       </c>
@@ -17161,20 +17161,20 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>153</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -17355,36 +17355,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -17550,36 +17550,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -17771,36 +17771,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -17984,36 +17984,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -18185,36 +18185,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -18403,24 +18403,24 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
     </row>
@@ -18429,24 +18429,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>
@@ -18624,36 +18624,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -18831,36 +18831,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -19026,36 +19026,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -19239,36 +19239,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -19446,36 +19446,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -19641,36 +19641,36 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
     </row>
     <row r="14" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -19855,24 +19855,24 @@
       <c r="E11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
     </row>
@@ -19881,24 +19881,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>
@@ -20092,10 +20092,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="D12" s="8">
         <v>0.80042009748954401</v>
       </c>
@@ -20104,10 +20104,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="42"/>
       <c r="D13" s="8">
         <v>0.84999993588744904</v>
       </c>
@@ -20116,8 +20116,8 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
       <c r="D14" s="8">
         <v>0.90042009748954399</v>
       </c>
@@ -20130,24 +20130,24 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="38"/>
+      <c r="B16" s="41"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="42"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
     </row>

</xml_diff>